<commit_message>
bug para o cloud.ia resolver
</commit_message>
<xml_diff>
--- a/public/data/fabricas/lider_fandom.xlsx
+++ b/public/data/fabricas/lider_fandom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="164">
   <si>
     <t xml:space="preserve">CATÁLOGO DE PRODUTOS — FANDOM BOX</t>
   </si>
@@ -37,21 +37,24 @@
     <t xml:space="preserve">Preço Unit. (R$)</t>
   </si>
   <si>
+    <t xml:space="preserve">Categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coleção</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho</t>
+  </si>
+  <si>
     <t xml:space="preserve">Descrição</t>
   </si>
   <si>
-    <t xml:space="preserve">Coleção</t>
-  </si>
-  <si>
     <t xml:space="preserve">Material</t>
   </si>
   <si>
     <t xml:space="preserve">Idade Recomendada</t>
   </si>
   <si>
-    <t xml:space="preserve">Tamanho Embalagem</t>
-  </si>
-  <si>
     <t xml:space="preserve">Embalagem</t>
   </si>
   <si>
@@ -67,21 +70,24 @@
     <t xml:space="preserve">ROBIN JOVEM TITAS</t>
   </si>
   <si>
+    <t xml:space="preserve">Fandom Box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jovens Titãs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 x 10 x 16 cm</t>
+  </si>
+  <si>
     <t xml:space="preserve">O grupo de heróis adolescentes mais adorado por todas as gerações chega ao universo do Fandom Box. Com estilo único e articulado, os personagens desta coleção são fabricados 100% no Brasil. O produto vem em uma embalagem transparente exclusiva (a box) que funciona como um verdadeiro case do Fandom.</t>
   </si>
   <si>
-    <t xml:space="preserve">Jovens Titãs</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vinil atóxico</t>
   </si>
   <si>
     <t xml:space="preserve">+3 anos</t>
   </si>
   <si>
-    <t xml:space="preserve">13 x 10 x 16 cm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Plástico rígido transparente (Box)</t>
   </si>
   <si>
@@ -145,12 +151,12 @@
     <t xml:space="preserve">MONICA TM</t>
   </si>
   <si>
+    <t xml:space="preserve">Turma da Mônica</t>
+  </si>
+  <si>
     <t xml:space="preserve">A turminha mais amada do Brasil ganha seu espaço no universo do Fandom Box Baby, encantando todos com seu estilo fofinho, cute cute e traços mais delicados. Esta linha conta com 5 bonecos colecionáveis de alta qualidade, com articulações e estilo único, produção 100% brasileira.</t>
   </si>
   <si>
-    <t xml:space="preserve">Turma da Mônica</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://images.tcdn.com.br/img/img_prod/727032/fandom_box_turma_da_monica_baby_monica_1461_2_fc9233c276573148d1a60aaadadae2dd.jpg</t>
   </si>
   <si>
@@ -211,12 +217,12 @@
     <t xml:space="preserve">SR DOS ANEIS - GOLLUM</t>
   </si>
   <si>
+    <t xml:space="preserve">Senhor dos Anéis</t>
+  </si>
+  <si>
     <t xml:space="preserve">Do fundo das cavernas e dos ecos da Montanha da Perdição, Gollum surge com toda a inquietude e contradição que fizeram dele uma das figuras mais inesquecíveis da Terra-média.</t>
   </si>
   <si>
-    <t xml:space="preserve">Senhor dos Anéis</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://images.tcdn.com.br/img/img_prod/727032/fandom_box_senhor_dos_anis_gollum_2_20260212143538_858f19a3123d.png</t>
   </si>
   <si>
@@ -304,12 +310,12 @@
     <t xml:space="preserve">MONICA FRIENDS</t>
   </si>
   <si>
+    <t xml:space="preserve">Friends</t>
+  </si>
+  <si>
     <t xml:space="preserve">Do seriado de TV de grande sucesso ao universo do Fandom Box, chegou a vez dos Friends ganharem uma coleção exclusiva! A coleção é composta por 6 bonecos com articulações, representando os principais integrantes desse grupo, fabricados com qualidade, estilo e expressões únicas.</t>
   </si>
   <si>
-    <t xml:space="preserve">Friends</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://images.tcdn.com.br/img/img_prod/727032/fandom_box_friends_monica_1415_1_7fcec4d2d2971e66775a33524708cfe0.jpg</t>
   </si>
   <si>
@@ -382,12 +388,12 @@
     <t xml:space="preserve">SCOOBY DOO SD</t>
   </si>
   <si>
+    <t xml:space="preserve">Scooby-Doo!</t>
+  </si>
+  <si>
     <t xml:space="preserve">O grupo de detetives mais atrapalhados e icônicos, chega com tudo no universo do Fandom Box. Os 5 bonecos desta coleção possuem articulações e estilo único, trazendo de volta a nostalgia deste desenho que encanta gerações.</t>
   </si>
   <si>
-    <t xml:space="preserve">Scooby-Doo!</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://res.cloudinary.com/dfkebb4ds/image/upload/v1773081441/scooby_olawti.jpg</t>
   </si>
   <si>
@@ -448,12 +454,12 @@
     <t xml:space="preserve">PERNALONGA LOONEY</t>
   </si>
   <si>
+    <t xml:space="preserve">Looney Tunes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Os personagens do Looney Tunes chegam ao universo do Fandom Box Classic nos lembrando que todos temos um lado fã para nos orgulhar. Com características fiéis aos 5 principais personagens da animação, fabricada totalmente no Brasil, com articulações nos bonecos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Looney Tunes</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://res.cloudinary.com/dfkebb4ds/image/upload/v1773080376/pernalonga_kkdtn5.jpg</t>
   </si>
   <si>
@@ -506,9 +512,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://res.cloudinary.com/dfkebb4ds/image/upload/v1773080395/FRAJOLA_2_rxbljw.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL GERAL</t>
   </si>
 </sst>
 </file>
@@ -597,7 +600,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -612,19 +615,6 @@
       <right style="thin">
         <color rgb="FFBBBBBB"/>
       </right>
-      <top style="thin">
-        <color rgb="FFBBBBBB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBBBBBB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin">
-        <color rgb="FFBBBBBB"/>
-      </left>
-      <right/>
       <top style="thin">
         <color rgb="FFBBBBBB"/>
       </top>
@@ -659,7 +649,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -694,14 +684,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -781,20 +763,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -812,6 +794,7 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -850,13 +833,16 @@
       <c r="L2" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>4</v>
@@ -865,36 +851,39 @@
         <v>72.04</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>21</v>
+        <v>21</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>4</v>
@@ -902,37 +891,40 @@
       <c r="D4" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>15</v>
+      <c r="E4" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>25</v>
+        <v>21</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>4</v>
@@ -941,36 +933,39 @@
         <v>72.04</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>29</v>
+        <v>21</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>4</v>
@@ -978,37 +973,40 @@
       <c r="D6" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>15</v>
+      <c r="E6" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>33</v>
+        <v>21</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>4</v>
@@ -1017,36 +1015,39 @@
         <v>72.04</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>37</v>
+        <v>21</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>4</v>
@@ -1054,37 +1055,40 @@
       <c r="D8" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>41</v>
+      <c r="E8" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>43</v>
+        <v>21</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>4</v>
@@ -1093,36 +1097,39 @@
         <v>72.04</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>44</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>47</v>
+        <v>21</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>4</v>
@@ -1130,37 +1137,40 @@
       <c r="D10" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>41</v>
+      <c r="E10" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>51</v>
+        <v>21</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>4</v>
@@ -1169,36 +1179,39 @@
         <v>72.04</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>44</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>55</v>
+        <v>21</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>4</v>
@@ -1206,37 +1219,40 @@
       <c r="D12" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>41</v>
+      <c r="E12" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>59</v>
+        <v>21</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>4</v>
@@ -1245,36 +1261,39 @@
         <v>72.04</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>66</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>65</v>
+        <v>21</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>4</v>
@@ -1282,37 +1301,40 @@
       <c r="D14" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>69</v>
+      <c r="E14" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>71</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>70</v>
+        <v>21</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>4</v>
@@ -1321,36 +1343,39 @@
         <v>72.04</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>75</v>
+        <v>21</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L15" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>4</v>
@@ -1358,37 +1383,40 @@
       <c r="D16" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>79</v>
+      <c r="E16" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>81</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>80</v>
+        <v>21</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>4</v>
@@ -1397,36 +1425,39 @@
         <v>72.04</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>84</v>
+        <v>16</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>86</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>85</v>
+        <v>21</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>4</v>
@@ -1434,37 +1465,40 @@
       <c r="D18" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>89</v>
+      <c r="E18" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>91</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>90</v>
+        <v>21</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>4</v>
@@ -1473,36 +1507,39 @@
         <v>72.04</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K19" s="4" t="s">
-        <v>96</v>
+        <v>21</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>4</v>
@@ -1510,37 +1547,40 @@
       <c r="D20" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>94</v>
+      <c r="E20" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>100</v>
+        <v>21</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>4</v>
@@ -1549,36 +1589,39 @@
         <v>72.04</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>104</v>
+        <v>21</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>4</v>
@@ -1586,37 +1629,40 @@
       <c r="D22" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>94</v>
+      <c r="E22" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K22" s="7" t="s">
-        <v>108</v>
+        <v>21</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C23" s="3" t="n">
         <v>4</v>
@@ -1625,36 +1671,39 @@
         <v>72.04</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>94</v>
+        <v>16</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>112</v>
+        <v>21</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>4</v>
@@ -1662,37 +1711,40 @@
       <c r="D24" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>94</v>
+      <c r="E24" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>97</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K24" s="7" t="s">
-        <v>116</v>
+        <v>21</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L24" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>4</v>
@@ -1701,36 +1753,39 @@
         <v>72.04</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>123</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K25" s="4" t="s">
-        <v>122</v>
+        <v>21</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
+      </c>
+      <c r="M25" s="4" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>4</v>
@@ -1738,37 +1793,40 @@
       <c r="D26" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>120</v>
+      <c r="E26" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>123</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>126</v>
+        <v>21</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>4</v>
@@ -1777,36 +1835,39 @@
         <v>72.04</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>123</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>130</v>
+        <v>21</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>4</v>
@@ -1814,37 +1875,40 @@
       <c r="D28" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>120</v>
+      <c r="E28" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>123</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>134</v>
+        <v>21</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L28" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C29" s="3" t="n">
         <v>4</v>
@@ -1853,36 +1917,39 @@
         <v>72.04</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>123</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K29" s="4" t="s">
-        <v>138</v>
+        <v>21</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
+      </c>
+      <c r="M29" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>4</v>
@@ -1890,37 +1957,40 @@
       <c r="D30" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>142</v>
+      <c r="E30" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K30" s="7" t="s">
-        <v>144</v>
+        <v>21</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="M30" s="7" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C31" s="3" t="n">
         <v>4</v>
@@ -1929,36 +1999,39 @@
         <v>72.04</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>142</v>
+        <v>16</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K31" s="4" t="s">
-        <v>148</v>
+        <v>21</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L31" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
+      </c>
+      <c r="M31" s="4" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>4</v>
@@ -1966,37 +2039,40 @@
       <c r="D32" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E32" s="7" t="s">
-        <v>142</v>
+      <c r="E32" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K32" s="7" t="s">
-        <v>152</v>
+        <v>21</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
+      </c>
+      <c r="M32" s="7" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C33" s="3" t="n">
         <v>4</v>
@@ -2005,36 +2081,39 @@
         <v>72.04</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>142</v>
+        <v>16</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>145</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K33" s="4" t="s">
-        <v>156</v>
+        <v>21</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>4</v>
@@ -2042,54 +2121,37 @@
       <c r="D34" s="8" t="n">
         <v>72.04</v>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>142</v>
+      <c r="E34" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>18</v>
+        <v>18</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="K34" s="7" t="s">
-        <v>160</v>
+        <v>21</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9" t="n">
-        <f aca="false">SUM(C3:C34)</f>
-        <v>128</v>
-      </c>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="M34" s="7" t="s">
+        <v>163</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A35:J35"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>